<commit_message>
Replace with latest from Sharepoint
</commit_message>
<xml_diff>
--- a/input/requirements/PatientSummary.xlsx
+++ b/input/requirements/PatientSummary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\NL-PS-IG\input\requirements\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nictiznl.sharepoint.com/sites/Zib-transitiecommunity/Gedeelde documenten/Architectuur/Werkgroepen ZIBS 2.0 Implementatie/Informatiestandaarden/NL-PS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3673" documentId="8_{E18A75D0-0588-41D5-84D2-F29C11C8C8B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A6029D8-12F4-4F8A-8D56-FD790CBB3DCE}"/>
+  <xr:revisionPtr revIDLastSave="3784" documentId="8_{E18A75D0-0588-41D5-84D2-F29C11C8C8B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E11E35D5-17B6-4B55-B107-F48A18AD68CC}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
   </bookViews>
   <sheets>
     <sheet name="Concept" sheetId="12" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="286">
   <si>
     <t>Veld</t>
   </si>
@@ -77,15 +77,13 @@
     <t>Alias(sen)</t>
   </si>
   <si>
-    <t>BGZ, spoedsamenvatting</t>
+    <t>Gezondheidsoverzicht, Patiëntoverzicht</t>
   </si>
   <si>
     <t>Juist gebruik</t>
   </si>
   <si>
-    <t>Patient Summary usecase situaties: implementation guide link 
-- spoedsamenvatting
--BGZ aanvragen</t>
+    <t>Ter ondersteuning van de zorgverlener in geval van noodsituaties, ongeplande en geplande zorg, zowel in eigen land als in het buitenland</t>
   </si>
   <si>
     <t>Onjuist gebruik</t>
@@ -166,6 +164,9 @@
     <t>Nummer</t>
   </si>
   <si>
+    <t>Label</t>
+  </si>
+  <si>
     <t>Naam</t>
   </si>
   <si>
@@ -190,6 +191,27 @@
     <t>NLPS-001</t>
   </si>
   <si>
+    <t>EU:</t>
+  </si>
+  <si>
+    <t>Header</t>
+  </si>
+  <si>
+    <t>Document header, containing the basic metadata for this NL-PS.</t>
+  </si>
+  <si>
+    <t>sectie/hoofdstuk aanduiding die de metadata bevat</t>
+  </si>
+  <si>
+    <t>1..1</t>
+  </si>
+  <si>
+    <t>Xt-EHR LIM 1.0.0 Document</t>
+  </si>
+  <si>
+    <t>NLPS-002</t>
+  </si>
+  <si>
     <t>subject</t>
   </si>
   <si>
@@ -199,13 +221,7 @@
     <t>(reference Patient)</t>
   </si>
   <si>
-    <t>1..1</t>
-  </si>
-  <si>
-    <t>Xt-EHR LIM 1.0.0 Document</t>
-  </si>
-  <si>
-    <t>NLPS-002</t>
+    <t>NLPS-003</t>
   </si>
   <si>
     <t>identifier</t>
@@ -220,7 +236,7 @@
     <t>Zie discussie</t>
   </si>
   <si>
-    <t>NLPS-003</t>
+    <t>NLPS-004</t>
   </si>
   <si>
     <t>author</t>
@@ -235,7 +251,7 @@
     <t>1..*</t>
   </si>
   <si>
-    <t>NLPS-004</t>
+    <t>NLPS-005</t>
   </si>
   <si>
     <t>date</t>
@@ -247,7 +263,7 @@
     <t>(dateTime)</t>
   </si>
   <si>
-    <t>NLPS-005</t>
+    <t>NLPS-006</t>
   </si>
   <si>
     <t>status</t>
@@ -259,7 +275,7 @@
     <t>(coding)</t>
   </si>
   <si>
-    <t>NLPS-006</t>
+    <t>NLPS-007</t>
   </si>
   <si>
     <t>language</t>
@@ -274,7 +290,7 @@
     <t>0..1</t>
   </si>
   <si>
-    <t>NLPS-007</t>
+    <t>NLPS-008</t>
   </si>
   <si>
     <t xml:space="preserve">type </t>
@@ -289,7 +305,7 @@
     <t>Xt-EHR LIM 1.0.0 EHDSPatientSummary</t>
   </si>
   <si>
-    <t>NLPS-008</t>
+    <t>NLPS-009</t>
   </si>
   <si>
     <t>title</t>
@@ -304,7 +320,7 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>NLPS-009</t>
+    <t>NLPS-010</t>
   </si>
   <si>
     <t>period</t>
@@ -313,7 +329,7 @@
     <t>Time period of information covered in the document</t>
   </si>
   <si>
-    <t>NLPS-010</t>
+    <t>NLPS-011</t>
   </si>
   <si>
     <t>version</t>
@@ -325,7 +341,7 @@
     <t>(string)</t>
   </si>
   <si>
-    <t>NLPS-011</t>
+    <t>NLPS-012</t>
   </si>
   <si>
     <t>attestation</t>
@@ -334,13 +350,13 @@
     <t>Document attestation details</t>
   </si>
   <si>
-    <t>(container)</t>
-  </si>
-  <si>
-    <t>0..*</t>
-  </si>
-  <si>
-    <t>NLPS-012</t>
+    <t>bestaat altijd uit een attester, datum en mode</t>
+  </si>
+  <si>
+    <t>0..* mag afwezig zijn, mag vaker voorkomen.</t>
+  </si>
+  <si>
+    <t>NLPS-013</t>
   </si>
   <si>
     <t>attester[x]</t>
@@ -352,31 +368,34 @@
     <t>(reference PractitionerRole, Practitioner, Device)</t>
   </si>
   <si>
-    <t>NLPS-013</t>
-  </si>
-  <si>
-    <t>mode</t>
+    <t>per authenticatie 1..1 vullen. als Attestion aanwezig, dan moet dit element ook aanwezig zijn</t>
+  </si>
+  <si>
+    <t>NLPS-014</t>
+  </si>
+  <si>
+    <t>mode of attestation</t>
   </si>
   <si>
     <t>Indicates the level of authority of the attestation. The type of attestation the authenticator offers.</t>
   </si>
   <si>
-    <t>coded https://hl7.org/fhir/R4/valueset-composition-attestation-mode.html</t>
+    <t>(coded) https://hl7.org/fhir/R4/valueset-composition-attestation-mode.html</t>
   </si>
   <si>
     <t>Base FHIR R4</t>
   </si>
   <si>
-    <t>NLPS-014</t>
-  </si>
-  <si>
-    <t>dateTime</t>
+    <t>NLPS-015</t>
+  </si>
+  <si>
+    <t>dateTime of attestation</t>
   </si>
   <si>
     <t>Date and time of the approval of the document by Attester</t>
   </si>
   <si>
-    <t>NLPS-015</t>
+    <t>NLPS-016</t>
   </si>
   <si>
     <t>legalAuthentication</t>
@@ -385,7 +404,10 @@
     <t>Document legal authentication details</t>
   </si>
   <si>
-    <t>NLPS-016</t>
+    <t>bestaat altijd uit een legalAuthenticator, datum en mode</t>
+  </si>
+  <si>
+    <t>NLPS-017</t>
   </si>
   <si>
     <t>legalAuthenticator</t>
@@ -397,16 +419,28 @@
     <t>(reference PractitionerRole, Practitioner, Organization)</t>
   </si>
   <si>
-    <t>NLPS-017</t>
+    <t>per authenticatie 1..1 vullen. als legalAuthentication aanwezig, dan moet dit element ook aanwezig zijn</t>
+  </si>
+  <si>
+    <t>NLPS-018</t>
+  </si>
+  <si>
+    <t>dateTime of legal authentication</t>
   </si>
   <si>
     <t>Date and time when the document was authorised</t>
   </si>
   <si>
-    <t>NLPS-018</t>
-  </si>
-  <si>
     <t>NLPS-019</t>
+  </si>
+  <si>
+    <t>mode of legal authentication</t>
+  </si>
+  <si>
+    <t>(coded) https://hl7.org/fhir/R4/valueset-composition-attestation-mode.html met required Pattern: legal</t>
+  </si>
+  <si>
+    <t>NLPS-020</t>
   </si>
   <si>
     <t>eventType</t>
@@ -419,7 +453,10 @@
 Binding Description: (preferred): LOINC, SNOMED CT, dicom-cid-33-Modality</t>
   </si>
   <si>
-    <t>NLPS-020</t>
+    <t>0..*</t>
+  </si>
+  <si>
+    <t>NLPS-021</t>
   </si>
   <si>
     <t>ServiceSpecialty</t>
@@ -432,7 +469,7 @@
 Binding Description: (preferred) SNOMED CT</t>
   </si>
   <si>
-    <t>NLPS-021</t>
+    <t>NLPS-022</t>
   </si>
   <si>
     <t>custodian</t>
@@ -444,7 +481,7 @@
     <t>(reference Organization)</t>
   </si>
   <si>
-    <t>NLPS-022</t>
+    <t>NLPS-023</t>
   </si>
   <si>
     <t>presentedForm</t>
@@ -460,7 +497,7 @@
 In EHDS is de conceptmapping "no-map" naar composition en alleen in Diagnostic report resource mag het voorkomen. Ook in de PS conceptmap is deze afwezig</t>
   </si>
   <si>
-    <t>NLPS-023</t>
+    <t>NLPS-024</t>
   </si>
   <si>
     <t>allergiesAndIntolerances</t>
@@ -472,7 +509,7 @@
     <t>HumanReadable (Text), Machine readable (code)</t>
   </si>
   <si>
-    <t>NLPS-023.1</t>
+    <t>NLPS-025</t>
   </si>
   <si>
     <t>generatedNarrative</t>
@@ -488,7 +525,7 @@
 Conditie in samenhang met entry. een van de twee moet aanwezig zijn</t>
   </si>
   <si>
-    <t>NLPS-023.2</t>
+    <t>NLPS-026</t>
   </si>
   <si>
     <t>Entry.AllergyIntolerance</t>
@@ -506,7 +543,7 @@
 A section SHALL at least have an generatedNarrative or entry (cmp-1)</t>
   </si>
   <si>
-    <t>NLPS-023.3</t>
+    <t>NLPS-027</t>
   </si>
   <si>
     <t>emptyReason</t>
@@ -523,7 +560,7 @@
 A section SHALL NOT have an emptyReason and entry at the same time. (cmp-2)</t>
   </si>
   <si>
-    <t>NLPS-023.3.1</t>
+    <t>NLPS-028</t>
   </si>
   <si>
     <t xml:space="preserve">Reason for absence of data: indicates whether the person is known to have no allergies </t>
@@ -532,7 +569,7 @@
     <t xml:space="preserve">in case if the person is known to have no allergies </t>
   </si>
   <si>
-    <t>NLPS-023.3.2</t>
+    <t>NLPS-029</t>
   </si>
   <si>
     <t>Reason for absence of data: the data is considered incomplete</t>
@@ -541,7 +578,7 @@
     <t>in case if the data is considered incomplete</t>
   </si>
   <si>
-    <t>NLPS-023.4</t>
+    <t>NLPS-030</t>
   </si>
   <si>
     <t>note</t>
@@ -550,7 +587,7 @@
     <t>Free text notes by the health professional</t>
   </si>
   <si>
-    <t>NLPS-023.5</t>
+    <t>NLPS-031</t>
   </si>
   <si>
     <t>code</t>
@@ -569,7 +606,7 @@
     <t>komt vanuit de IPS</t>
   </si>
   <si>
-    <t>NLPS-023.6</t>
+    <t>NLPS-032</t>
   </si>
   <si>
     <t>The label for this particular section. This will be part of the rendered content for the document, and is often used to build a table of contents.</t>
@@ -578,7 +615,7 @@
     <t>Title (Text)</t>
   </si>
   <si>
-    <t>NLPS-024</t>
+    <t>NLPS-033</t>
   </si>
   <si>
     <t>problems</t>
@@ -587,10 +624,10 @@
     <t>Section: Problems. Human readable denominator to identify the topic of this section.</t>
   </si>
   <si>
-    <t>NLPS-024.1</t>
-  </si>
-  <si>
-    <t>NLPS-024.2</t>
+    <t>NLPS-034</t>
+  </si>
+  <si>
+    <t>NLPS-035</t>
   </si>
   <si>
     <t>problem</t>
@@ -602,26 +639,26 @@
     <t>(reference EHDSCondition)</t>
   </si>
   <si>
-    <t>NLPS-024.3</t>
+    <t>NLPS-036</t>
   </si>
   <si>
     <t>Use if no conditions are listed</t>
   </si>
   <si>
-    <t>NLPS-024.4</t>
-  </si>
-  <si>
-    <t>NLPS-024.5</t>
+    <t>NLPS-037</t>
+  </si>
+  <si>
+    <t>NLPS-038</t>
   </si>
   <si>
     <t>Binding: DocumentSectionCodes (example)
 fixed value: LOINC 11450-4</t>
   </si>
   <si>
-    <t>NLPS-024.6</t>
-  </si>
-  <si>
-    <t>NLPS-025</t>
+    <t>NLPS-039</t>
+  </si>
+  <si>
+    <t>NLPS-040</t>
   </si>
   <si>
     <t>medicationSummary</t>
@@ -630,10 +667,10 @@
     <t>Section: Medication Summary. Human readable denominator to identify the topic of this section.</t>
   </si>
   <si>
-    <t>NLPS-025.1</t>
-  </si>
-  <si>
-    <t>NLPS-025.2</t>
+    <t>NLPS-041</t>
+  </si>
+  <si>
+    <t>NLPS-042</t>
   </si>
   <si>
     <t>medicationUse</t>
@@ -645,26 +682,26 @@
     <t>(reference EHDSMedicationUse) MP9 blok</t>
   </si>
   <si>
-    <t>NLPS-025.3</t>
+    <t>NLPS-043</t>
   </si>
   <si>
     <t>Use if no medicines are listed</t>
   </si>
   <si>
-    <t>NLPS-025.4</t>
-  </si>
-  <si>
-    <t>NLPS-025.5</t>
+    <t>NLPS-044</t>
+  </si>
+  <si>
+    <t>NLPS-045</t>
   </si>
   <si>
     <t>Binding: DocumentSectionCodes (example)
 fixed value: LOINC 10160-0</t>
   </si>
   <si>
-    <t>NLPS-025.6</t>
-  </si>
-  <si>
-    <t>NLPS-026</t>
+    <t>NLPS-046</t>
+  </si>
+  <si>
+    <t>NLPS-047</t>
   </si>
   <si>
     <t>medicalDevicesAndImplants</t>
@@ -673,10 +710,10 @@
     <t>Section: Medical devices and implants. Human readable denominator to identify the topic of this section.</t>
   </si>
   <si>
-    <t>NLPS-026.1</t>
-  </si>
-  <si>
-    <t>NLPS-026.2</t>
+    <t>NLPS-048</t>
+  </si>
+  <si>
+    <t>NLPS-049</t>
   </si>
   <si>
     <t>deviceUse</t>
@@ -688,26 +725,26 @@
     <t>(reference EHDSDeviceUse)</t>
   </si>
   <si>
-    <t>NLPS-026.3</t>
+    <t>NLPS-050</t>
   </si>
   <si>
     <t>Use if no medical devices or implants are listed</t>
   </si>
   <si>
-    <t>NLPS-026.4</t>
-  </si>
-  <si>
-    <t>NLPS-026.5</t>
+    <t>NLPS-051</t>
+  </si>
+  <si>
+    <t>NLPS-052</t>
   </si>
   <si>
     <t>Binding: DocumentSectionCodes (example)
 fixed value: LOINC 46264-8</t>
   </si>
   <si>
-    <t>NLPS-026.6</t>
-  </si>
-  <si>
-    <t>NLPS-027</t>
+    <t>NLPS-053</t>
+  </si>
+  <si>
+    <t>NLPS-054</t>
   </si>
   <si>
     <t>Procedures</t>
@@ -716,13 +753,13 @@
     <t>Section: Procedures. Human readable denominator to identify the topic of this section.</t>
   </si>
   <si>
-    <t>NLPS-027.1</t>
+    <t>NLPS-055</t>
   </si>
   <si>
     <t>Narrative (Text+code)</t>
   </si>
   <si>
-    <t>NLPS-027.2</t>
+    <t>NLPS-056</t>
   </si>
   <si>
     <t>procedure</t>
@@ -734,23 +771,23 @@
     <t>(reference EHDSProcedure)</t>
   </si>
   <si>
-    <t>NLPS-027.3</t>
+    <t>NLPS-057</t>
   </si>
   <si>
     <t>Use if no procedures are listed</t>
   </si>
   <si>
-    <t>NLPS-027.4</t>
-  </si>
-  <si>
-    <t>NLPS-027.5</t>
+    <t>NLPS-058</t>
+  </si>
+  <si>
+    <t>NLPS-059</t>
   </si>
   <si>
     <t>Binding: DocumentSectionCodes (example)
 fixed value: LOINC 47519-4</t>
   </si>
   <si>
-    <t>NLPS-027.6</t>
+    <t>NLPS-060</t>
   </si>
   <si>
     <t>Actie</t>
@@ -813,13 +850,13 @@
     <t>EmptyReason LIM</t>
   </si>
   <si>
-    <t>In LIM wordt er bij elke verplicht concept een optie gegeven voor EmptyReason, als je geen informatie hebt. Hier zien wij nog geen oplossing voor in de EPS. Wij verwachten dat hier in FHIR wel gewerkt kan worden met de standaard Emptyreason. Maar in de EPS missen we nog deze uitleg</t>
-  </si>
-  <si>
-    <t>In EU-PS wordt dit in de EU-PS-Composition afgevangen met het element emptyReason bij 3 van de 4 verplichte elementen. Dit zal dan ook in het GBB-Composition met obligations moeten komen. Ook in het GBB-Composition moet dit functioneel gemaakt worden met de zelfde waardelijst.</t>
-  </si>
-  <si>
-    <t>nog een fhir ticket aanmaken, dat ze niet consistent zijn met Xt-EHR</t>
+    <t>In LIM wordt er bij elke verplicht concept een optie gegeven voor EmptyReason, als je geen informatie hebt. Hier zien wij nog geen consistente oplossing voor in de EPS profiel. Wij verwachten dat hier in FHIR wel gewerkt kan worden met de standaard Emptyreason bij sections. Maar de constraint ips-comp-1 is inconsistent.</t>
+  </si>
+  <si>
+    <t>In EU-PS wordt dit in de EU-PS-Composition afgevangen met het element emptyReason bij 3 van de 5 verplichte elementen. In het GBB-Composition en NL-PS maken wij dit wel consistent met obligations en constraints voor alle verplichte concepten. Procedures en DeviceUse</t>
+  </si>
+  <si>
+    <t>nog een fhir ticket aanmaken, ips-coms-1 en de obligations bij Procedure en DeviceUse dat ze niet consistent zijn met Xt-EHR</t>
   </si>
   <si>
     <t>Kardinaliteit LIM vs FHIR EPS</t>
@@ -857,6 +894,9 @@
     <t>presented form</t>
   </si>
   <si>
+    <t>In LIM EU wordt presented forms grevraagd. in FHIR profiel van EU-PS is daar geen oplossing voor gevonden. Daar staat "no-map" richitng de composition</t>
+  </si>
+  <si>
     <t>repeating sections in compositions</t>
   </si>
   <si>
@@ -864,13 +904,28 @@
   </si>
   <si>
     <t>Informatiebehoefte_Composition.xlsx</t>
+  </si>
+  <si>
+    <t>Coding sections</t>
+  </si>
+  <si>
+    <t>In FHIR profiel is minimaal een fixed value per section-code verwacht. Nog uitzoeken hoe dit ook in Afsprakenmodel kan werken. Ook nog opnemen als "minimaal de fixed value + uitleg over watr voor andere codes hier ook mogen komen"</t>
+  </si>
+  <si>
+    <t>GeneratedNartive (Lim), Section.text (FHIR profiel)</t>
+  </si>
+  <si>
+    <t>In de LIM is er een kardinaliteit van 0..1 terwijl in het FHIR profiel op 1..1 staat</t>
+  </si>
+  <si>
+    <t>Ticket aangemaakt: https://jira.hl7.org/browse/FHIR-58821</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1091,9 +1146,9 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="20">
     <dxf>
       <font>
         <color rgb="FF000000"/>
@@ -1239,6 +1294,9 @@
       <fill>
         <patternFill patternType="none"/>
       </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1736,10 +1794,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ADCD9434-A4C3-4190-B536-08977257489F}" name="Tabel1" displayName="Tabel1" ref="A2:H61" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17" tableBorderDxfId="16">
-  <autoFilter ref="A2:H61" xr:uid="{ADCD9434-A4C3-4190-B536-08977257489F}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{9AEF381A-368B-41A9-8CC6-43DE2198447B}" name="Nummer" dataDxfId="15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ADCD9434-A4C3-4190-B536-08977257489F}" name="Tabel1" displayName="Tabel1" ref="A2:I62" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18" tableBorderDxfId="17">
+  <autoFilter ref="A2:I62" xr:uid="{ADCD9434-A4C3-4190-B536-08977257489F}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{9AEF381A-368B-41A9-8CC6-43DE2198447B}" name="Nummer" dataDxfId="16"/>
+    <tableColumn id="10" xr3:uid="{E69112D2-CDD7-44F2-9D15-783070E07781}" name="Label" dataDxfId="15"/>
     <tableColumn id="2" xr3:uid="{8DD74A41-15FD-4EC5-A225-EAEB16110411}" name="Naam" dataDxfId="14"/>
     <tableColumn id="3" xr3:uid="{97B49655-5A49-4567-AC26-589A9901D374}" name="Omschrijving" dataDxfId="13"/>
     <tableColumn id="4" xr3:uid="{5F654189-A8EA-48BB-B7B3-64E2B20A1ED4}" name="Variabiliteit" dataDxfId="12"/>
@@ -2085,16 +2144,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACC5AB7C-ED78-4367-9B8E-D6DDDB80D1B1}">
   <dimension ref="A1:D24"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="62.44140625" customWidth="1"/>
+    <col min="2" max="2" width="62.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="190.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="190.5" customHeight="1">
       <c r="A1" s="20"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4">
       <c r="A2" s="21" t="s">
         <v>0</v>
       </c>
@@ -2102,7 +2161,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="75">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2112,7 +2171,7 @@
       <c r="C3" s="1"/>
       <c r="D3" s="6"/>
     </row>
-    <row r="4" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="30">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -2122,7 +2181,7 @@
       <c r="C4" s="1"/>
       <c r="D4" s="6"/>
     </row>
-    <row r="5" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="60">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -2132,7 +2191,7 @@
       <c r="C5" s="1"/>
       <c r="D5" s="6"/>
     </row>
-    <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="15.75">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2142,7 +2201,7 @@
       <c r="C6" s="1"/>
       <c r="D6" s="6"/>
     </row>
-    <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="15.75">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -2151,7 +2210,7 @@
       </c>
       <c r="D7" s="7"/>
     </row>
-    <row r="8" spans="1:4" ht="63" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" ht="63" customHeight="1">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -2161,7 +2220,7 @@
       <c r="C8" s="1"/>
       <c r="D8" s="9"/>
     </row>
-    <row r="9" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" ht="15.75">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -2171,7 +2230,7 @@
       <c r="C9" s="1"/>
       <c r="D9" s="7"/>
     </row>
-    <row r="10" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="15.75">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -2181,7 +2240,7 @@
       <c r="C10" s="1"/>
       <c r="D10" s="6"/>
     </row>
-    <row r="11" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" ht="15.75">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -2191,56 +2250,56 @@
       <c r="C11" s="1"/>
       <c r="D11" s="6"/>
     </row>
-    <row r="12" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" ht="15.75">
       <c r="C12" s="1"/>
       <c r="D12" s="6"/>
     </row>
-    <row r="13" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" ht="15.75">
       <c r="B13" s="4"/>
       <c r="C13" s="17"/>
       <c r="D13" s="6"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4">
       <c r="B14" s="18"/>
       <c r="C14" s="17"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4">
       <c r="B15" s="18"/>
       <c r="C15" s="17"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4">
       <c r="B16" s="4"/>
       <c r="C16" s="17"/>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:3">
       <c r="B17" s="4"/>
       <c r="C17" s="17"/>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:3">
       <c r="B18" s="4"/>
       <c r="C18" s="1"/>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:3">
       <c r="B19" s="4"/>
       <c r="C19" s="17"/>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:3">
       <c r="B20" s="4"/>
       <c r="C20" s="17"/>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:3">
       <c r="B21" s="1"/>
       <c r="C21" s="17"/>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:3">
       <c r="B22" s="4"/>
       <c r="C22" s="17"/>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:3">
       <c r="B23" s="4"/>
       <c r="C23" s="17"/>
     </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:3">
       <c r="B24" s="4"/>
       <c r="C24" s="1"/>
     </row>
@@ -2253,15 +2312,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C76C4CDD-06CC-4FA3-8CD3-C85562DBC01E}">
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="28.109375" customWidth="1"/>
-    <col min="2" max="2" width="53.109375" customWidth="1"/>
-    <col min="3" max="3" width="19.5546875" customWidth="1"/>
-    <col min="4" max="4" width="43.109375" customWidth="1"/>
+    <col min="1" max="1" width="28.140625" customWidth="1"/>
+    <col min="2" max="2" width="53.140625" customWidth="1"/>
+    <col min="3" max="3" width="19.5703125" customWidth="1"/>
+    <col min="4" max="4" width="43.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4">
       <c r="A1" s="22" t="s">
         <v>19</v>
       </c>
@@ -2275,7 +2334,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4">
       <c r="A2" s="17" t="s">
         <v>23</v>
       </c>
@@ -2284,7 +2343,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4">
       <c r="A3" s="17" t="s">
         <v>25</v>
       </c>
@@ -2293,7 +2352,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4">
       <c r="A4" s="17" t="s">
         <v>26</v>
       </c>
@@ -2302,7 +2361,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4">
       <c r="A5" s="17" t="s">
         <v>27</v>
       </c>
@@ -2311,7 +2370,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4">
       <c r="A6" s="17" t="s">
         <v>28</v>
       </c>
@@ -2320,7 +2379,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
         <v>27</v>
       </c>
@@ -2329,7 +2388,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4">
       <c r="A8" s="17" t="s">
         <v>28</v>
       </c>
@@ -2338,7 +2397,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" ht="29.25">
       <c r="A9" s="17" t="s">
         <v>29</v>
       </c>
@@ -2349,7 +2408,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="29.25">
       <c r="A10" s="17" t="s">
         <v>32</v>
       </c>
@@ -2360,7 +2419,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4">
       <c r="A11" s="17" t="s">
         <v>34</v>
       </c>
@@ -2371,7 +2430,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4">
       <c r="A12" s="17" t="s">
         <v>36</v>
       </c>
@@ -2382,7 +2441,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4">
       <c r="A13" s="17" t="s">
         <v>38</v>
       </c>
@@ -2391,7 +2450,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4">
       <c r="A14" s="17" t="s">
         <v>38</v>
       </c>
@@ -2413,22 +2472,23 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD25B5EA-7FC2-4A85-8C2E-196DE7DE592E}">
-  <dimension ref="A2:I61"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:K62"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.6640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="26.44140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="78.44140625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="33" style="3" customWidth="1"/>
-    <col min="5" max="5" width="36.88671875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="27.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="35.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="44.88671875" style="3" customWidth="1"/>
-    <col min="9" max="9" width="0" style="2" hidden="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.109375" style="2" hidden="1"/>
+    <col min="1" max="2" width="13.7109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="26.42578125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="78.42578125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="33" style="3" customWidth="1"/>
+    <col min="6" max="6" width="36.85546875" style="3" customWidth="1"/>
+    <col min="7" max="7" width="27.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="35.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="44.85546875" style="3" customWidth="1"/>
+    <col min="10" max="10" width="0" style="2" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="0" style="2" hidden="1"/>
+    <col min="12" max="16384" width="9.140625" style="2" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:8" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" s="27" customFormat="1">
       <c r="A2" s="25" t="s">
         <v>39</v>
       </c>
@@ -2438,75 +2498,77 @@
       <c r="C2" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="D2" s="26" t="s">
+      <c r="D2" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="E2" s="25" t="s">
+      <c r="E2" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="F2" s="25" t="s">
+      <c r="F2" s="26" t="s">
         <v>44</v>
       </c>
       <c r="G2" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="H2" s="26" t="s">
+      <c r="H2" s="25" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I2" s="26" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" s="27" customFormat="1" ht="29.25">
       <c r="A3" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C3" s="3" t="s">
         <v>49</v>
       </c>
+      <c r="C3" s="2" t="s">
+        <v>50</v>
+      </c>
       <c r="D3" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="I3" s="3"/>
+      <c r="J3" s="2"/>
+    </row>
+    <row r="4" spans="1:10">
       <c r="A4" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="G4" s="24"/>
+      <c r="H4" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="F4" s="24"/>
-      <c r="G4" s="24" t="s">
-        <v>52</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:10" ht="19.5" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B5" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>60</v>
       </c>
       <c r="D5" s="3" t="s">
@@ -2515,1201 +2577,1230 @@
       <c r="E5" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="F5" s="24"/>
-      <c r="G5" s="24" t="s">
-        <v>52</v>
-      </c>
-      <c r="H5" s="2"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F5" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="29.25">
       <c r="A6" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B6" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>65</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="G6" s="24" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E6" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="I6" s="2"/>
+    </row>
+    <row r="7" spans="1:10">
       <c r="A7" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C7" s="3" t="s">
         <v>69</v>
       </c>
+      <c r="C7" s="2" t="s">
+        <v>70</v>
+      </c>
       <c r="D7" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="G7" s="24" t="s">
-        <v>52</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H7" s="24" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
       <c r="A8" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C8" s="3" t="s">
         <v>73</v>
       </c>
+      <c r="C8" s="2" t="s">
+        <v>74</v>
+      </c>
       <c r="D8" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E8" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="G8" s="24" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E8" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H8" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="29.25">
       <c r="A9" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B9" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="G9" s="24" t="s">
+      <c r="E9" s="3" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="F9" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H9" s="24" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="29.25">
       <c r="A10" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B10" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>83</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="G10" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H10" s="3" t="s">
+      <c r="E10" s="3" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H10" s="24" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="43.5">
       <c r="A11" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H11" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="B11" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="G11" s="24" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I11" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
       <c r="A12" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>93</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="G12" s="24" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+        <v>94</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H12" s="24" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="29.25">
       <c r="A13" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C13" s="3" t="s">
         <v>95</v>
       </c>
+      <c r="C13" s="2" t="s">
+        <v>96</v>
+      </c>
       <c r="D13" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="E13" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="G13" s="24" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E13" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H13" s="24" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="29.25">
       <c r="A14" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B14" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>100</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="G14" s="24" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E14" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="H14" s="24" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="43.5">
       <c r="A15" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="B15" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="H15" s="24" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="43.5">
+      <c r="A16" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="I16" s="11"/>
+    </row>
+    <row r="17" spans="1:9" ht="43.5">
+      <c r="A17" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="H17" s="24" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="29.25">
+      <c r="A18" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="F18" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="C15" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="H15" s="11"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="G16" s="24" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="B17" s="2" t="s">
+      <c r="H18" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="I18" s="2"/>
+    </row>
+    <row r="19" spans="1:9" ht="60.75" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="H19" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="I19" s="2"/>
+    </row>
+    <row r="20" spans="1:9" ht="43.5">
+      <c r="A20" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="H20" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="I20" s="2"/>
+    </row>
+    <row r="21" spans="1:9" ht="43.5">
+      <c r="A21" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="D21" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="C17" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="G17" s="24"/>
-      <c r="H17" s="2"/>
-    </row>
-    <row r="18" spans="1:8" ht="60.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
+      <c r="E21" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="G18" s="24" t="s">
-        <v>52</v>
-      </c>
-      <c r="H18" s="2"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="G19" s="24" t="s">
-        <v>52</v>
-      </c>
-      <c r="H19" s="2"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="B20" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="E20" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="H20" s="11"/>
-    </row>
-    <row r="21" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="G21" s="24" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I21" s="11"/>
+    </row>
+    <row r="22" spans="1:9" ht="57.75">
       <c r="A22" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>125</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>126</v>
+        <v>132</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>133</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="G22" s="24" t="s">
-        <v>52</v>
-      </c>
-      <c r="H22" s="2"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+        <v>134</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="H22" s="24" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="43.5">
       <c r="A23" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>130</v>
+        <v>137</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>138</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="G23" s="24" t="s">
-        <v>52</v>
-      </c>
-      <c r="H23" s="2"/>
-    </row>
-    <row r="24" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+        <v>139</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="H23" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="I23" s="2"/>
+    </row>
+    <row r="24" spans="1:9">
       <c r="A24" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>134</v>
+        <v>141</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>142</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="H24" s="2"/>
-    </row>
-    <row r="25" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>144</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H24" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="I24" s="2"/>
+    </row>
+    <row r="25" spans="1:9" ht="72.75">
       <c r="A25" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>139</v>
+        <v>145</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>146</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G25" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H25" s="2"/>
-    </row>
-    <row r="26" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+        <v>148</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="I25" s="2"/>
+    </row>
+    <row r="26" spans="1:9" ht="29.25">
       <c r="A26" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>143</v>
+        <v>150</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>151</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="G26" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H26" s="2"/>
-    </row>
-    <row r="27" spans="1:8" ht="157.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>153</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H26" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I26" s="2"/>
+    </row>
+    <row r="27" spans="1:9" ht="43.5">
       <c r="A27" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>148</v>
+        <v>154</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>155</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="G27" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H27" s="2"/>
-    </row>
-    <row r="28" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
+        <v>157</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="H27" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I27" s="2"/>
+    </row>
+    <row r="28" spans="1:9" ht="157.5" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C28" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="H28" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I28" s="2"/>
+    </row>
+    <row r="29" spans="1:9" ht="101.25">
+      <c r="A29" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="H29" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I29" s="2"/>
+    </row>
+    <row r="30" spans="1:9" ht="43.5">
+      <c r="A30" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="H30" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I30" s="2"/>
+    </row>
+    <row r="31" spans="1:9" ht="43.5">
+      <c r="A31" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="H31" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I31" s="2"/>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H32" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I32" s="2"/>
+    </row>
+    <row r="33" spans="1:9" ht="43.5">
+      <c r="A33" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H33" s="24" t="s">
+        <v>182</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="29.25">
+      <c r="A34" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H34" s="24" t="s">
+        <v>182</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="29.25">
+      <c r="A35" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="E35" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="D28" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="E28" s="3" t="s">
+      <c r="F35" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H35" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I35" s="2"/>
+    </row>
+    <row r="36" spans="1:9" ht="43.5">
+      <c r="A36" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="G28" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H28" s="2"/>
-    </row>
-    <row r="29" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A29" s="2" t="s">
+      <c r="D36" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C29" s="3" t="s">
+      <c r="E36" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="D29" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="E29" s="3" t="s">
+      <c r="F36" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="G29" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H29" s="2"/>
-    </row>
-    <row r="30" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A30" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="D30" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="G30" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H30" s="2"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A31" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="B31" s="2" t="s">
+      <c r="H36" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I36" s="2"/>
+    </row>
+    <row r="37" spans="1:9" ht="144.75">
+      <c r="A37" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F37" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="C31" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="D31" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="G31" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H31" s="2"/>
-    </row>
-    <row r="32" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
+      <c r="H37" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I37" s="2"/>
+    </row>
+    <row r="38" spans="1:9" ht="101.25">
+      <c r="A38" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="C32" s="3" t="s">
+      <c r="D38" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="E38" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="F38" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="E32" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G32" s="24" t="s">
-        <v>169</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A33" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="D33" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G33" s="24" t="s">
-        <v>169</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A34" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="C34" s="3" t="s">
+      <c r="H38" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I38" s="2"/>
+    </row>
+    <row r="39" spans="1:9">
+      <c r="A39" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="D34" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G34" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H34" s="2"/>
-    </row>
-    <row r="35" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A35" s="2" t="s">
+      <c r="D39" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="B35" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="G35" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H35" s="2"/>
-    </row>
-    <row r="36" spans="1:8" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A36" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="B36" s="2" t="s">
+      <c r="E39" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H39" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I39" s="2"/>
+    </row>
+    <row r="40" spans="1:9" ht="43.5">
+      <c r="A40" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="D40" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="D36" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="G36" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H36" s="2"/>
-    </row>
-    <row r="37" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A37" s="2" t="s">
+      <c r="E40" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H40" s="24" t="s">
         <v>182</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C37" s="2" t="s">
+      <c r="I40" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="D37" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="E37" s="3" t="s">
+    </row>
+    <row r="41" spans="1:9" ht="29.25">
+      <c r="A41" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H41" s="24" t="s">
+        <v>182</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="29.25">
+      <c r="A42" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H42" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I42" s="2"/>
+    </row>
+    <row r="43" spans="1:9" ht="43.5">
+      <c r="A43" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="G37" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H37" s="2"/>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A38" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="B38" s="2" t="s">
+      <c r="D43" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="H43" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I43" s="2"/>
+    </row>
+    <row r="44" spans="1:9" ht="144.75">
+      <c r="A44" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="E44" s="28" t="s">
+        <v>208</v>
+      </c>
+      <c r="F44" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="C38" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="D38" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="G38" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H38" s="2"/>
-    </row>
-    <row r="39" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A39" s="2" t="s">
+      <c r="H44" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I44" s="2"/>
+    </row>
+    <row r="45" spans="1:9" ht="101.25">
+      <c r="A45" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F45" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="H45" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I45" s="2"/>
+    </row>
+    <row r="46" spans="1:9">
+      <c r="A46" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F46" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H46" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I46" s="2"/>
+    </row>
+    <row r="47" spans="1:9" ht="43.5">
+      <c r="A47" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H47" s="24" t="s">
+        <v>182</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="29.25">
+      <c r="A48" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D48" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="B39" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="C39" s="3" t="s">
+      <c r="E48" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H48" s="24" t="s">
+        <v>182</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="29.25">
+      <c r="A49" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H49" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I49" s="2"/>
+    </row>
+    <row r="50" spans="1:9" ht="43.5">
+      <c r="A50" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="F50" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="H50" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I50" s="2"/>
+    </row>
+    <row r="51" spans="1:9" ht="144.75">
+      <c r="A51" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="F51" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="H51" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I51" s="2"/>
+    </row>
+    <row r="52" spans="1:9" ht="101.25">
+      <c r="A52" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="E52" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="F52" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="H52" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I52" s="2"/>
+    </row>
+    <row r="53" spans="1:9">
+      <c r="A53" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F53" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H53" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I53" s="2"/>
+    </row>
+    <row r="54" spans="1:9" ht="43.5">
+      <c r="A54" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="F54" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H54" s="24" t="s">
+        <v>182</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="29.25">
+      <c r="A55" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="E55" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="E39" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G39" s="24" t="s">
-        <v>169</v>
-      </c>
-      <c r="H39" s="2" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A40" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="D40" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G40" s="24" t="s">
-        <v>169</v>
-      </c>
-      <c r="H40" s="2" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A41" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="B41" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="D41" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="E41" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G41" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H41" s="2"/>
-    </row>
-    <row r="42" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A42" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="D42" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="G42" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H42" s="2"/>
-    </row>
-    <row r="43" spans="1:8" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A43" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="D43" s="28" t="s">
-        <v>195</v>
-      </c>
-      <c r="E43" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="G43" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H43" s="2"/>
-    </row>
-    <row r="44" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A44" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="D44" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="E44" s="3" t="s">
+      <c r="F55" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H55" s="24" t="s">
+        <v>182</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="29.25">
+      <c r="A56" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="F56" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H56" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I56" s="2"/>
+    </row>
+    <row r="57" spans="1:9" ht="43.5">
+      <c r="A57" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="C57" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="G44" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H44" s="2"/>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A45" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="B45" s="2" t="s">
+      <c r="D57" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="F57" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="H57" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I57" s="2"/>
+    </row>
+    <row r="58" spans="1:9" ht="144.75">
+      <c r="A58" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="F58" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="C45" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="D45" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="E45" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="G45" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H45" s="2"/>
-    </row>
-    <row r="46" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A46" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="C46" s="3" t="s">
+      <c r="H58" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I58" s="2"/>
+    </row>
+    <row r="59" spans="1:9" ht="101.25">
+      <c r="A59" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="E59" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="D46" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="E46" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G46" s="24" t="s">
-        <v>169</v>
-      </c>
-      <c r="H46" s="2" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A47" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="D47" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="E47" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G47" s="24" t="s">
-        <v>169</v>
-      </c>
-      <c r="H47" s="2" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A48" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="D48" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="E48" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G48" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H48" s="2"/>
-    </row>
-    <row r="49" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A49" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="D49" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="E49" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="G49" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H49" s="2"/>
-    </row>
-    <row r="50" spans="1:8" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A50" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>208</v>
-      </c>
-      <c r="D50" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="E50" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="G50" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H50" s="2"/>
-    </row>
-    <row r="51" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A51" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="D51" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="E51" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="G51" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H51" s="2"/>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A52" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="C52" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="D52" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="E52" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="G52" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H52" s="2"/>
-    </row>
-    <row r="53" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A53" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="C53" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="D53" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="E53" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G53" s="24" t="s">
-        <v>169</v>
-      </c>
-      <c r="H53" s="2" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A54" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C54" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="E54" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G54" s="24" t="s">
-        <v>169</v>
-      </c>
-      <c r="H54" s="2" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A55" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="B55" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="C55" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="D55" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="E55" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G55" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H55" s="2"/>
-    </row>
-    <row r="56" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A56" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="C56" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="D56" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="E56" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="G56" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H56" s="2"/>
-    </row>
-    <row r="57" spans="1:8" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A57" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="C57" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="D57" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="E57" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="G57" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H57" s="2"/>
-    </row>
-    <row r="58" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A58" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="B58" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="D58" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="E58" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="G58" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H58" s="2"/>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A59" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="C59" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="D59" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="E59" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="G59" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="H59" s="2"/>
-    </row>
-    <row r="60" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="F59" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="H59" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I59" s="2"/>
+    </row>
+    <row r="60" spans="1:9">
       <c r="A60" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="C60" s="3" t="s">
-        <v>167</v>
+        <v>240</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>176</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>229</v>
+        <v>177</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G60" s="24" t="s">
-        <v>169</v>
-      </c>
-      <c r="H60" s="2" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="61" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>98</v>
+      </c>
+      <c r="F60" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H60" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I60" s="2"/>
+    </row>
+    <row r="61" spans="1:9" ht="43.5">
       <c r="A61" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C61" s="3" t="s">
-        <v>172</v>
+        <v>241</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>179</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G61" s="29" t="s">
-        <v>169</v>
-      </c>
-      <c r="H61" s="2" t="s">
-        <v>170</v>
+        <v>242</v>
+      </c>
+      <c r="F61" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H61" s="24" t="s">
+        <v>182</v>
+      </c>
+      <c r="I61" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" ht="29.25">
+      <c r="A62" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="F62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H62" s="29" t="s">
+        <v>182</v>
+      </c>
+      <c r="I62" s="2" t="s">
+        <v>183</v>
       </c>
     </row>
   </sheetData>
@@ -3723,72 +3814,72 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECE81417-31BE-416B-8441-5485E15A4072}">
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.44140625" customWidth="1"/>
-    <col min="2" max="2" width="18.5546875" customWidth="1"/>
-    <col min="3" max="3" width="16.88671875" customWidth="1"/>
-    <col min="4" max="4" width="86.109375" customWidth="1"/>
-    <col min="5" max="5" width="16.5546875" customWidth="1"/>
-    <col min="6" max="6" width="16.44140625" customWidth="1"/>
-    <col min="7" max="7" width="41.5546875" customWidth="1"/>
+    <col min="1" max="1" width="19.42578125" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" customWidth="1"/>
+    <col min="4" max="4" width="86.140625" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" customWidth="1"/>
+    <col min="7" max="7" width="41.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="195.75" customHeight="1">
       <c r="A1" s="21" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="B1" s="21" t="s">
-        <v>232</v>
+        <v>245</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G1" s="21" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" s="23" t="s">
-        <v>233</v>
+        <v>246</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>235</v>
+        <v>248</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>236</v>
+        <v>249</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>237</v>
+        <v>250</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>240</v>
+        <v>253</v>
       </c>
       <c r="C3" t="s">
-        <v>241</v>
+        <v>254</v>
       </c>
       <c r="D3" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>
@@ -3800,9 +3891,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF34F478-5AEF-4FD0-9200-F4CED1FB07BC}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" ht="111" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="1" ht="111" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3812,104 +3903,104 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE3F362B-60AA-4A98-B52B-B8CA0A560EE5}">
   <dimension ref="A2:G65"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.88671875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="24.5546875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="21.44140625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="68.88671875" style="3" customWidth="1"/>
-    <col min="5" max="5" width="22.88671875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="50.44140625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="31.5546875" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="9.109375" style="2"/>
+    <col min="1" max="1" width="3.85546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="24.5703125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="21.42578125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="68.85546875" style="3" customWidth="1"/>
+    <col min="5" max="5" width="22.85546875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="50.42578125" style="3" customWidth="1"/>
+    <col min="7" max="7" width="31.5703125" style="2" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:7">
       <c r="B2" s="5" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.3">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7">
       <c r="B3" s="8" t="s">
-        <v>244</v>
+        <v>257</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>245</v>
+        <v>258</v>
       </c>
       <c r="D3" s="19" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>247</v>
+        <v>260</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="4" spans="2:7" ht="105.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" ht="105.75" customHeight="1">
       <c r="B4" s="12" t="s">
-        <v>250</v>
+        <v>263</v>
       </c>
       <c r="C4" s="11"/>
       <c r="D4" s="13" t="s">
-        <v>251</v>
+        <v>264</v>
       </c>
       <c r="E4" s="16"/>
       <c r="F4" s="12" t="s">
-        <v>252</v>
+        <v>265</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="5" spans="2:7" ht="140.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" ht="140.25" customHeight="1">
       <c r="B5" s="12" t="s">
-        <v>254</v>
+        <v>267</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="13" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="E5" s="11"/>
       <c r="F5" s="12" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
       <c r="G5" s="11"/>
     </row>
-    <row r="6" spans="2:7" ht="126" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:7" ht="126" customHeight="1">
       <c r="B6" s="12" t="s">
-        <v>257</v>
+        <v>270</v>
       </c>
       <c r="C6"/>
       <c r="D6" s="12" t="s">
-        <v>258</v>
+        <v>271</v>
       </c>
       <c r="E6" s="11"/>
       <c r="F6" s="12" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="G6" s="11"/>
     </row>
-    <row r="7" spans="2:7" ht="90.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:7" ht="140.25" customHeight="1">
       <c r="B7" s="12" t="s">
-        <v>260</v>
+        <v>273</v>
       </c>
       <c r="C7" s="11"/>
       <c r="D7" s="12" t="s">
-        <v>261</v>
+        <v>274</v>
       </c>
       <c r="E7" s="11"/>
       <c r="F7" s="12" t="s">
-        <v>262</v>
+        <v>275</v>
       </c>
       <c r="G7" s="11"/>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:7">
       <c r="B8" s="12" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
       <c r="C8" s="11"/>
       <c r="D8" s="12"/>
@@ -3917,19 +4008,21 @@
       <c r="F8" s="12"/>
       <c r="G8" s="11"/>
     </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:7" ht="29.25">
       <c r="B9" s="12" t="s">
-        <v>263</v>
+        <v>276</v>
       </c>
       <c r="C9" s="11"/>
-      <c r="D9" s="12"/>
+      <c r="D9" s="12" t="s">
+        <v>277</v>
+      </c>
       <c r="E9" s="11"/>
       <c r="F9" s="12"/>
       <c r="G9" s="11"/>
     </row>
-    <row r="10" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:7" ht="30">
       <c r="B10" s="12" t="s">
-        <v>264</v>
+        <v>278</v>
       </c>
       <c r="C10" s="11"/>
       <c r="D10" s="12"/>
@@ -3937,35 +4030,45 @@
       <c r="F10" s="12"/>
       <c r="G10" s="11"/>
     </row>
-    <row r="11" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:7" ht="29.25">
       <c r="B11" s="12" t="s">
-        <v>265</v>
+        <v>279</v>
       </c>
       <c r="C11" s="11"/>
       <c r="D11" s="18" t="s">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="E11" s="11"/>
       <c r="F11" s="12"/>
       <c r="G11" s="11"/>
     </row>
-    <row r="12" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="12"/>
+    <row r="12" spans="2:7" ht="57.75">
+      <c r="B12" s="12" t="s">
+        <v>281</v>
+      </c>
       <c r="C12" s="11"/>
-      <c r="D12" s="12"/>
+      <c r="D12" s="12" t="s">
+        <v>282</v>
+      </c>
       <c r="E12" s="11"/>
       <c r="F12" s="12"/>
       <c r="G12" s="11"/>
     </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B13" s="12"/>
+    <row r="13" spans="2:7" ht="29.25">
+      <c r="B13" s="12" t="s">
+        <v>283</v>
+      </c>
       <c r="C13" s="11"/>
-      <c r="D13" s="12"/>
+      <c r="D13" s="12" t="s">
+        <v>284</v>
+      </c>
       <c r="E13" s="11"/>
-      <c r="F13" s="12"/>
+      <c r="F13" s="12" t="s">
+        <v>285</v>
+      </c>
       <c r="G13" s="11"/>
     </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:7">
       <c r="B14" s="12"/>
       <c r="C14" s="11"/>
       <c r="D14" s="12"/>
@@ -3973,7 +4076,7 @@
       <c r="F14" s="12"/>
       <c r="G14" s="11"/>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:7">
       <c r="B15" s="12"/>
       <c r="C15" s="11"/>
       <c r="D15" s="12"/>
@@ -3981,7 +4084,7 @@
       <c r="F15" s="12"/>
       <c r="G15" s="11"/>
     </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:7">
       <c r="B16" s="12"/>
       <c r="C16" s="11"/>
       <c r="D16" s="12"/>
@@ -3989,7 +4092,7 @@
       <c r="F16" s="12"/>
       <c r="G16" s="11"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7">
       <c r="B17" s="12"/>
       <c r="C17" s="11"/>
       <c r="D17" s="12"/>
@@ -3997,152 +4100,152 @@
       <c r="F17" s="12"/>
       <c r="G17" s="11"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7">
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
       <c r="D18" s="19"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7">
       <c r="B19" s="3"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7">
       <c r="B20" s="3"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7">
       <c r="B21" s="3"/>
     </row>
-    <row r="22" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" ht="19.5" customHeight="1">
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
       <c r="D22" s="19"/>
     </row>
-    <row r="23" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" ht="19.5" customHeight="1">
       <c r="B23" s="3"/>
     </row>
-    <row r="24" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" ht="19.5" customHeight="1">
       <c r="B24" s="3"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7">
       <c r="B25" s="3"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7">
       <c r="B26" s="3"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7">
       <c r="A27" s="3"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7">
       <c r="A28" s="3"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7">
       <c r="A29" s="3"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7">
       <c r="A30" s="3"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7">
       <c r="A31" s="3"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7">
       <c r="A32" s="3"/>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:1">
       <c r="A33" s="3"/>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:1">
       <c r="A34" s="3"/>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:1">
       <c r="A35" s="3"/>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:1">
       <c r="A36" s="3"/>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:1">
       <c r="A37" s="3"/>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:1">
       <c r="A38" s="3"/>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:1">
       <c r="A39" s="3"/>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:1">
       <c r="A40" s="3"/>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:1">
       <c r="A41" s="3"/>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:1">
       <c r="A42" s="3"/>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:1">
       <c r="A43" s="3"/>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:1">
       <c r="A44" s="3"/>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:1">
       <c r="A45" s="3"/>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:1">
       <c r="A46" s="3"/>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:1">
       <c r="A47" s="3"/>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:1">
       <c r="A48" s="3"/>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:1">
       <c r="A49" s="3"/>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:1">
       <c r="A50" s="3"/>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:1">
       <c r="A51" s="3"/>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:1">
       <c r="A52" s="3"/>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:1">
       <c r="A53" s="3"/>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:1">
       <c r="A54" s="3"/>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:1">
       <c r="A55" s="3"/>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:1">
       <c r="A56" s="3"/>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:1">
       <c r="A57" s="3"/>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:1">
       <c r="A58" s="3"/>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:1">
       <c r="A59" s="3"/>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:1">
       <c r="A60" s="3"/>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:1">
       <c r="A61" s="3"/>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:1">
       <c r="A62" s="3"/>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:1">
       <c r="A63" s="3"/>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:1">
       <c r="A64" s="3"/>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:1">
       <c r="A65" s="3"/>
     </row>
   </sheetData>
@@ -4389,47 +4492,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C8F8F082-555E-4C95-A3AE-A46F01E1A119}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/DataMashup"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C8F8F082-555E-4C95-A3AE-A46F01E1A119}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C46046CF-AC59-4D6A-A325-5977C53DC9DA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
-    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C46046CF-AC59-4D6A-A325-5977C53DC9DA}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D91DC9B-0D61-455B-BDC2-0A4F28AD2AEE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
-    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D91DC9B-0D61-455B-BDC2-0A4F28AD2AEE}"/>
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}"/>
 </file>
</xml_diff>